<commit_message>
fix(quotation): adhere strictly to schematic drawing with 1 gateway
</commit_message>
<xml_diff>
--- a/ECO PRIME_Báo Giá Đồng Hồ Điện & CC2051_Pou Hui_20261021.xlsx
+++ b/ECO PRIME_Báo Giá Đồng Hồ Điện & CC2051_Pou Hui_20261021.xlsx
@@ -2722,12 +2722,12 @@
       </c>
       <c r="D16" s="113" t="inlineStr">
         <is>
-          <t>Bộ điều khiển/thu thập dữ liệu biên công nghiệp CC2051 (Edge Gateway), cổng RS-485 Modbus RTU thu thập tín hiệu từ các đồng hồ đo điện PM210, chuyển đổi sang Modbus TCP / MQTT qua cổng mạng RJ45 Ethernet, truyền dữ liệu liên tục về hệ thống EMS trung tâm.
-CC2051工業級邊緣計算與資料收集閘道器, 具備RS-485 Modbus RTU接口採集PM210電表數據, 經由RJ45以太網轉換為Modbus TCP/MQTT協議, 即時上傳至中央能源管理系統 (EMS)。</t>
+          <t>Bộ điều khiển/thu thập dữ liệu biên công nghiệp CC2051 (Edge Gateway), cổng RS-485 Modbus RTU thu thập tín hiệu từ 4 đồng hồ đo điện PM210-4-V của 4 trạm biến áp, chuyển đổi sang Modbus TCP / MQTT qua cổng mạng RJ45 Ethernet kết nối LAN Switch về EMS trung tâm.
+CC2051工業級邊緣計算與資料收集閘道器, 具備RS-485 Modbus RTU接口採集4座變電站PM210電表數據, 經由RJ45以太網轉換為Modbus TCP/MQTT協議, 經由LAN Switch即時上傳至中央能源管理系統 (EMS)。</t>
         </is>
       </c>
       <c r="E16" s="114" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F16" s="115" t="n"/>
       <c r="G16" s="116">

</xml_diff>

<commit_message>
fix(eco-prime): bundle 24vdc power supply into gateway cc2051 item
</commit_message>
<xml_diff>
--- a/ECO PRIME_Báo Giá Đồng Hồ Điện & CC2051_Pou Hui_20261021.xlsx
+++ b/ECO PRIME_Báo Giá Đồng Hồ Điện & CC2051_Pou Hui_20261021.xlsx
@@ -9,7 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PouHui" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'PouHui'!$A$1:$H$28</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'PouHui'!$A$1:$H$27</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -1368,7 +1368,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="161">
+  <cellXfs count="155">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -1730,31 +1730,10 @@
     <xf numFmtId="168" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="170" fontId="71" fillId="10" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="5">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="176" fontId="71" fillId="10" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="5">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="71" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="71" fillId="10" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="71" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="71" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="71" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="174" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="3">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="72" fillId="0" borderId="40" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1762,8 +1741,13 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="43" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="44" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="51" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="73" fillId="0" borderId="45" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="174" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="51" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="73" fillId="4" borderId="45" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="174" fontId="74" fillId="0" borderId="45" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1775,38 +1759,38 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="53" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="54" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="55" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="73" fillId="0" borderId="47" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="73" fillId="4" borderId="47" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="174" fontId="74" fillId="0" borderId="47" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="74" fillId="0" borderId="48" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="74" fillId="0" borderId="48" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="177" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="75" fillId="0" borderId="59" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
+    <xf numFmtId="0" fontId="75" fillId="4" borderId="59" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="60" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="61" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="76" fillId="0" borderId="64" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
+    <xf numFmtId="0" fontId="76" fillId="4" borderId="64" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="65" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="77" fillId="0" borderId="72" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
+    <xf numFmtId="0" fontId="77" fillId="4" borderId="72" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="73" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="78" fillId="0" borderId="75" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
+    <xf numFmtId="0" fontId="78" fillId="4" borderId="75" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="76" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="70" fillId="0" borderId="75" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
+    <xf numFmtId="0" fontId="53" fillId="4" borderId="75" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="74" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="79" fillId="0" borderId="77" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="79" fillId="4" borderId="77" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="78" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -2704,26 +2688,26 @@
         <v/>
       </c>
     </row>
-    <row r="16" ht="211" customFormat="1" customHeight="1" s="6">
+    <row r="16" ht="250" customFormat="1" customHeight="1" s="6">
       <c r="A16" s="110" t="n">
         <v>4</v>
       </c>
       <c r="B16" s="111" t="inlineStr">
         <is>
-          <t>Gateway thu thập dữ liệu CC2051
-CC2051 工業級資料收集閘道器</t>
+          <t>Gateway thu thập dữ liệu CC2051 (kèm bộ nguồn 24VDC)
+CC2051 工業級資料收集閘道器 (含24VDC電源供應器)</t>
         </is>
       </c>
       <c r="C16" s="112" t="inlineStr">
         <is>
-          <t>Gateway thu thập dữ liệu
-數據採集網關</t>
+          <t>Gateway &amp; Nguồn
+數據閘道器及電源</t>
         </is>
       </c>
       <c r="D16" s="113" t="inlineStr">
         <is>
-          <t>Bộ điều khiển/thu thập dữ liệu biên công nghiệp CC2051 (Edge Gateway), cổng RS-485 Modbus RTU thu thập tín hiệu từ 4 đồng hồ đo điện PM210-4-V của 4 trạm biến áp, chuyển đổi sang Modbus TCP / MQTT qua cổng mạng RJ45 Ethernet kết nối LAN Switch về EMS trung tâm.
-CC2051工業級邊緣計算與資料收集閘道器, 具備RS-485 Modbus RTU接口採集4座變電站PM210電表數據, 經由RJ45以太網轉換為Modbus TCP/MQTT協議, 經由LAN Switch即時上傳至中央能源管理系統 (EMS)。</t>
+          <t>Bộ điều khiển/thu thập dữ liệu biên công nghiệp CC2051 (Edge Gateway) kèm bộ nguồn công nghiệp Din-rail 24VDC chuyên dụng, cổng RS-485 Modbus RTU thu thập tín hiệu từ 4 đồng hồ đo điện PM210-4-V của 4 trạm biến áp, chuyển đổi sang Modbus TCP / MQTT qua cổng mạng RJ45 Ethernet kết nối LAN Switch về EMS trung tâm.
+CC2051工業級邊緣計算與資料收集閘道器 (含專用導軌式24VDC開關電源供應器), 具備RS-485 Modbus RTU接口採集4座變電站PM210電表數據, 經由RJ45以太網轉換為Modbus TCP/MQTT協議, 經由LAN Switch即時上傳至中央能源管理系統 (EMS)。</t>
         </is>
       </c>
       <c r="E16" s="114" t="n">
@@ -2759,30 +2743,30 @@
         <v/>
       </c>
     </row>
-    <row r="17" ht="172" customFormat="1" customHeight="1" s="6">
+    <row r="17" ht="152.5" customFormat="1" customHeight="1" s="6">
       <c r="A17" s="110" t="n">
         <v>5</v>
       </c>
       <c r="B17" s="111" t="inlineStr">
         <is>
-          <t>Bộ nguồn công nghiệp 24VDC (PW)
-工業級電源供應器 (PW)</t>
+          <t>Bộ chia mạng công nghiệp 5-Port
+工業級5埠乙太網交換機 (LAN SWITCH)</t>
         </is>
       </c>
       <c r="C17" s="112" t="inlineStr">
         <is>
-          <t>Nguồn cấp công nghiệp
-電源供應器</t>
+          <t>Thiết bị mạng
+網絡設備</t>
         </is>
       </c>
       <c r="D17" s="113" t="inlineStr">
         <is>
-          <t>Bộ nguồn công nghiệp gắn Din-rail Meanwell/tương đương, điện áp vào dải rộng AC 85~265V, đầu ra DC 24V ổn định, chống sét lan truyền và quá tải, cấp nguồn liên tục cho Gateway CC2051 và đồng hồ PM210. 1 bộ / trạm biến áp.
-工業級導軌式開關電源供應器, 寬電壓輸入 AC 85~265V, 輸出 DC 24V 穩定電源, 具備過載與防雷保護, 為 PM210 電表及 CC2051 閘道器供電。每座變電站1台。</t>
+          <t>Switch mạng công nghiệp 5 cổng RJ45 10/100Mbps gắn thanh ray, vỏ kim loại chuẩn công nghiệp chống nhiễu điện từ, kết nối truyền dữ liệu từ Gateway CC2051 về mạng nội bộ LAN nhà máy.
+工業級5埠 10/100Mbps 導軌式交換機, 金屬抗干擾外殼, 適用於工廠高壓變電站環境, 將 CC2051 網關連接至廠區局域網 (LAN)。</t>
         </is>
       </c>
       <c r="E17" s="114" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F17" s="115" t="n"/>
       <c r="G17" s="116">
@@ -2814,78 +2798,23 @@
         <v/>
       </c>
     </row>
-    <row r="18" ht="152.5" customFormat="1" customHeight="1" s="6">
+    <row r="18" ht="211" customFormat="1" customHeight="1" s="6">
       <c r="A18" s="110" t="n">
         <v>6</v>
       </c>
       <c r="B18" s="111" t="inlineStr">
         <is>
-          <t>Bộ chia mạng công nghiệp 5-Port
-工業級5埠乙太網交換機 (LAN SWITCH)</t>
-        </is>
-      </c>
-      <c r="C18" s="112" t="inlineStr">
-        <is>
-          <t>Thiết bị mạng
-網絡設備</t>
-        </is>
-      </c>
-      <c r="D18" s="113" t="inlineStr">
-        <is>
-          <t>Switch mạng công nghiệp 5 cổng RJ45 10/100Mbps gắn thanh ray, vỏ kim loại chuẩn công nghiệp chống nhiễu điện từ, kết nối truyền dữ liệu từ các Gateway CC2051 về mạng nội bộ LAN nhà máy.
-工業級5埠 10/100Mbps 導軌式交換機, 金屬抗干擾外殼, 適用於工廠高壓變電站環境, 將 CC2051 網關連接至廠區局域網 (LAN)。</t>
-        </is>
-      </c>
-      <c r="E18" s="121" t="n">
-        <v>1</v>
-      </c>
-      <c r="F18" s="115" t="n"/>
-      <c r="G18" s="116">
-        <f>F18*E18</f>
-        <v/>
-      </c>
-      <c r="H18" s="117">
-        <f>G18*H12</f>
-        <v/>
-      </c>
-      <c r="J18" s="122" t="n"/>
-      <c r="K18" s="54" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="L18" s="119">
-        <f>J18*K18</f>
-        <v/>
-      </c>
-      <c r="M18">
-        <f>J18*0.07</f>
-        <v/>
-      </c>
-      <c r="N18" s="119">
-        <f>J18+L18+M18</f>
-        <v/>
-      </c>
-      <c r="O18" s="119">
-        <f>N18*E18</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19" ht="211" customFormat="1" customHeight="1" s="6">
-      <c r="A19" s="110" t="n">
-        <v>7</v>
-      </c>
-      <c r="B19" s="111" t="inlineStr">
-        <is>
           <t>Cáp mạng Cat6, cáp RS485 &amp; Vật tư phụ
 網絡線 Cat.6、RS485通訊線及安裝輔材</t>
         </is>
       </c>
-      <c r="C19" s="112" t="inlineStr">
+      <c r="C18" s="112" t="inlineStr">
         <is>
           <t>Vật tư phụ
 輔助材料</t>
         </is>
       </c>
-      <c r="D19" s="113" t="inlineStr">
+      <c r="D18" s="113" t="inlineStr">
         <is>
           <t>Bao gồm nội dung 內容包含:
 - Cáp mạng Cat6: 網絡線 Category 6 UTP Cable, 4-Pair
@@ -2894,56 +2823,56 @@
 - Đầu cosse bọc cách điện, nhãn đánh dấu dây cáp và toàn bộ phụ kiện đấu nối 冷壓端子、電纜號碼管及全套配線輔材。</t>
         </is>
       </c>
-      <c r="E19" s="123" t="n">
+      <c r="E18" s="121" t="n">
         <v>1</v>
       </c>
-      <c r="F19" s="115" t="n"/>
-      <c r="G19" s="116">
-        <f>F19*E19</f>
-        <v/>
-      </c>
-      <c r="H19" s="117">
-        <f>G19*H12</f>
-        <v/>
-      </c>
-      <c r="J19" s="122" t="n"/>
-      <c r="K19" s="54" t="n">
+      <c r="F18" s="115" t="n"/>
+      <c r="G18" s="116">
+        <f>F18*E18</f>
+        <v/>
+      </c>
+      <c r="H18" s="117">
+        <f>G18*H12</f>
+        <v/>
+      </c>
+      <c r="J18" s="122" t="n"/>
+      <c r="K18" s="54" t="n">
         <v>0.08</v>
       </c>
-      <c r="L19" s="119">
-        <f>J19*K19</f>
-        <v/>
-      </c>
-      <c r="M19">
-        <f>J19*0.07</f>
-        <v/>
-      </c>
-      <c r="N19" s="119">
-        <f>J19+L19+M19</f>
-        <v/>
-      </c>
-      <c r="O19" s="119">
-        <f>N19*E19</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20" ht="211" customHeight="1" thickBot="1">
-      <c r="A20" s="124" t="n">
-        <v>8</v>
-      </c>
-      <c r="B20" s="111" t="inlineStr">
+      <c r="L18" s="119">
+        <f>J18*K18</f>
+        <v/>
+      </c>
+      <c r="M18">
+        <f>J18*0.07</f>
+        <v/>
+      </c>
+      <c r="N18" s="119">
+        <f>J18+L18+M18</f>
+        <v/>
+      </c>
+      <c r="O18" s="119">
+        <f>N18*E18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="211" customFormat="1" customHeight="1" s="6">
+      <c r="A19" s="110" t="n">
+        <v>7</v>
+      </c>
+      <c r="B19" s="111" t="inlineStr">
         <is>
           <t>Chi phí thi công
 施工費</t>
         </is>
       </c>
-      <c r="C20" s="112" t="inlineStr">
+      <c r="C19" s="112" t="inlineStr">
         <is>
           <t>Chi phí thi công
 施工費</t>
         </is>
       </c>
-      <c r="D20" s="113" t="inlineStr">
+      <c r="D19" s="113" t="inlineStr">
         <is>
           <t>Bao gồm nội dung 內容包含:
 - Cài đặt hệ thống 系統設定
@@ -2954,177 +2883,178 @@
 - Chi phí đi lại, giàn giáo, dụng cụ an toàn 交通費、鷹架、工安器具...</t>
         </is>
       </c>
-      <c r="E20" s="125" t="n">
+      <c r="E19" s="121" t="n">
         <v>1</v>
       </c>
-      <c r="F20" s="126" t="n"/>
-      <c r="G20" s="127">
-        <f>F20*E20</f>
-        <v/>
-      </c>
-      <c r="H20" s="128">
-        <f>G20*H12</f>
-        <v/>
-      </c>
-      <c r="K20" t="n">
+      <c r="F19" s="115" t="n"/>
+      <c r="G19" s="116">
+        <f>F19*E19</f>
+        <v/>
+      </c>
+      <c r="H19" s="117">
+        <f>G19*H12</f>
+        <v/>
+      </c>
+      <c r="J19" s="122" t="n"/>
+      <c r="K19" s="54" t="n">
         <v>0.08</v>
       </c>
-      <c r="L20">
-        <f>J20*K20</f>
-        <v/>
-      </c>
-      <c r="M20">
-        <f>J20*0.07</f>
-        <v/>
-      </c>
-      <c r="N20" s="73">
-        <f>J20+L20+M20</f>
-        <v/>
-      </c>
-      <c r="O20" s="129">
-        <f>N20*E20</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="130" t="inlineStr">
+      <c r="L19" s="119">
+        <f>J19*K19</f>
+        <v/>
+      </c>
+      <c r="M19">
+        <f>J19*0.07</f>
+        <v/>
+      </c>
+      <c r="N19" s="119">
+        <f>J19+L19+M19</f>
+        <v/>
+      </c>
+      <c r="O19" s="119">
+        <f>N19*E19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1" thickBot="1">
+      <c r="A20" s="123" t="inlineStr">
         <is>
           <t>以下空白</t>
         </is>
       </c>
-      <c r="B21" s="131" t="n"/>
-      <c r="C21" s="131" t="n"/>
-      <c r="D21" s="131" t="n"/>
-      <c r="E21" s="131" t="n"/>
-      <c r="F21" s="131" t="n"/>
-      <c r="G21" s="131" t="n"/>
-      <c r="H21" s="132" t="n"/>
+      <c r="B20" s="124" t="n"/>
+      <c r="C20" s="124" t="n"/>
+      <c r="D20" s="124" t="n"/>
+      <c r="E20" s="124" t="n"/>
+      <c r="F20" s="124" t="n"/>
+      <c r="G20" s="124" t="n"/>
+      <c r="H20" s="125" t="n"/>
+      <c r="N20" s="73" t="inlineStr">
+        <is>
+          <t>合計成本</t>
+        </is>
+      </c>
+      <c r="O20" s="126">
+        <f>SUM(O13:O19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="38" customHeight="1">
+      <c r="A21" s="127" t="n"/>
+      <c r="F21" s="128" t="inlineStr">
+        <is>
+          <t>Tạm tính 小計</t>
+        </is>
+      </c>
+      <c r="G21" s="129">
+        <f>SUM(G13:G19)</f>
+        <v/>
+      </c>
+      <c r="H21" s="130">
+        <f>G21*H12</f>
+        <v/>
+      </c>
       <c r="N21" s="73" t="inlineStr">
         <is>
+          <t>合計成本</t>
+        </is>
+      </c>
+      <c r="O21" s="126">
+        <f>SUM(O13:O19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="38" customHeight="1">
+      <c r="A22" s="131" t="n"/>
+      <c r="F22" s="128" t="inlineStr">
+        <is>
+          <t>Thuế VAT 8% 增值稅</t>
+        </is>
+      </c>
+      <c r="G22" s="129">
+        <f>G21*0.08</f>
+        <v/>
+      </c>
+      <c r="H22" s="130">
+        <f>H21*0.08</f>
+        <v/>
+      </c>
+      <c r="N22" s="1" t="inlineStr">
+        <is>
           <t>利潤</t>
         </is>
       </c>
-      <c r="O21" s="129">
-        <f>G21-O20</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22" ht="38" customHeight="1">
-      <c r="A22" s="133" t="n"/>
-      <c r="F22" s="134" t="inlineStr">
-        <is>
-          <t>Tạm tính 小計</t>
-        </is>
-      </c>
-      <c r="G22" s="135">
-        <f>SUM(G13:G20)</f>
-        <v/>
-      </c>
-      <c r="H22" s="136">
-        <f>G22*H12</f>
-        <v/>
-      </c>
-      <c r="N22" s="1" t="inlineStr">
-        <is>
-          <t>合計成本</t>
-        </is>
-      </c>
       <c r="O22" s="54">
-        <f>SUM(O13:O20)</f>
+        <f>G21-O21</f>
         <v/>
       </c>
     </row>
     <row r="23" ht="38" customHeight="1" thickBot="1">
-      <c r="A23" s="137" t="n"/>
+      <c r="A23" s="132" t="n"/>
+      <c r="B23" s="133" t="n"/>
+      <c r="C23" s="133" t="n"/>
+      <c r="D23" s="133" t="n"/>
+      <c r="E23" s="133" t="n"/>
       <c r="F23" s="134" t="inlineStr">
         <is>
-          <t>Thuế VAT 8% 增值稅</t>
+          <t>Tổng cộng 總金額</t>
         </is>
       </c>
       <c r="G23" s="135">
-        <f>G22*0.08</f>
+        <f>G21*1.08</f>
         <v/>
       </c>
       <c r="H23" s="136">
-        <f>H22*0.08</f>
+        <f>H21*1.08</f>
         <v/>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>利潤</t>
-        </is>
-      </c>
-      <c r="O23">
-        <f>G22-O22</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24" ht="38" customHeight="1">
-      <c r="A24" s="138" t="n"/>
+          <t>% 利潤</t>
+        </is>
+      </c>
+      <c r="O23" s="137">
+        <f>O22/G21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="24" customHeight="1">
+      <c r="A24" s="138" t="inlineStr">
+        <is>
+          <t>※客戶確認 Xác nhận khách hàng</t>
+        </is>
+      </c>
       <c r="B24" s="139" t="n"/>
-      <c r="C24" s="139" t="n"/>
-      <c r="D24" s="139" t="n"/>
+      <c r="C24" s="140" t="n"/>
+      <c r="D24" s="141" t="inlineStr">
+        <is>
+          <t>◆ 備註聲明</t>
+        </is>
+      </c>
       <c r="E24" s="139" t="n"/>
-      <c r="F24" s="140" t="inlineStr">
-        <is>
-          <t>Tổng cộng 總金額</t>
-        </is>
-      </c>
-      <c r="G24" s="141">
-        <f>G22*1.08</f>
-        <v/>
-      </c>
-      <c r="H24" s="142">
-        <f>H22*1.08</f>
-        <v/>
-      </c>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t>% 利潤</t>
-        </is>
-      </c>
-      <c r="O24" s="143">
-        <f>O23/G22</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25" ht="24" customHeight="1">
-      <c r="A25" s="144" t="inlineStr">
-        <is>
-          <t>※客戶確認 Xác nhận khách hàng</t>
-        </is>
-      </c>
-      <c r="B25" s="145" t="n"/>
-      <c r="C25" s="146" t="n"/>
-      <c r="D25" s="147" t="inlineStr">
-        <is>
-          <t>◆ 備註聲明</t>
-        </is>
-      </c>
-      <c r="E25" s="145" t="n"/>
-      <c r="F25" s="145" t="n"/>
-      <c r="G25" s="145" t="n"/>
-      <c r="H25" s="148" t="n"/>
-    </row>
-    <row r="26" ht="54" customHeight="1">
-      <c r="A26" s="149" t="inlineStr">
+      <c r="F24" s="139" t="n"/>
+      <c r="G24" s="139" t="n"/>
+      <c r="H24" s="142" t="n"/>
+    </row>
+    <row r="25" ht="54" customHeight="1">
+      <c r="A25" s="143" t="inlineStr">
         <is>
           <t>（請簽名用印） Chữ ký và con dấu</t>
         </is>
       </c>
-      <c r="C26" s="150" t="n"/>
-      <c r="D26" s="151" t="inlineStr">
+      <c r="C25" s="144" t="n"/>
+      <c r="D25" s="145" t="inlineStr">
         <is>
           <t>1. 以上報價交期：報價單簽回後，另日程安排後回覆；
    Thời gian giao hàng của báo giá trên: sau khi báo giá được ký và gửi lại, lịch trình cụ thể sẽ được thông báo sau;</t>
         </is>
       </c>
-      <c r="H26" s="152" t="n"/>
-    </row>
-    <row r="27" ht="54" customHeight="1" thickBot="1">
-      <c r="A27" s="137" t="n"/>
-      <c r="C27" s="150" t="n"/>
-      <c r="D27" s="153" t="inlineStr">
+      <c r="H25" s="146" t="n"/>
+    </row>
+    <row r="26" ht="54" customHeight="1">
+      <c r="A26" s="131" t="n"/>
+      <c r="C26" s="144" t="n"/>
+      <c r="D26" s="147" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -3166,65 +3096,66 @@
           </r>
         </is>
       </c>
-      <c r="H27" s="152" t="n"/>
-    </row>
-    <row r="28" ht="58" customHeight="1">
-      <c r="A28" s="138" t="n"/>
-      <c r="B28" s="139" t="n"/>
-      <c r="C28" s="154" t="n"/>
-      <c r="D28" s="155" t="inlineStr">
+      <c r="H26" s="146" t="n"/>
+    </row>
+    <row r="27" ht="58" customHeight="1" thickBot="1">
+      <c r="A27" s="132" t="n"/>
+      <c r="B27" s="133" t="n"/>
+      <c r="C27" s="148" t="n"/>
+      <c r="D27" s="149" t="inlineStr">
         <is>
           <t>3. 付款方式 : 訂金 35%、 交貨 55%、驗收 10% TT30Day。
      Điều khoản thanh toán:  [Đặt cọc: 35%, Khi giao hàng: 55%, Sau khi nghiệm thu: Thanh toán 10% còn lại theo điều khoản TT 30 ngày (TT30 Days).]</t>
         </is>
       </c>
-      <c r="E28" s="139" t="n"/>
-      <c r="F28" s="139" t="n"/>
-      <c r="G28" s="139" t="n"/>
-      <c r="H28" s="156" t="n"/>
-    </row>
+      <c r="E27" s="133" t="n"/>
+      <c r="F27" s="133" t="n"/>
+      <c r="G27" s="133" t="n"/>
+      <c r="H27" s="150" t="n"/>
+    </row>
+    <row r="28"/>
     <row r="29"/>
     <row r="32">
-      <c r="G32" s="157" t="n"/>
+      <c r="G32" s="151" t="n"/>
     </row>
     <row r="33">
-      <c r="G33" s="158" t="n"/>
+      <c r="G33" s="152" t="n"/>
     </row>
     <row r="34">
-      <c r="G34" s="157" t="n"/>
+      <c r="G34" s="151" t="n"/>
     </row>
     <row r="35">
       <c r="F35" s="21" t="n"/>
-      <c r="G35" s="157" t="n"/>
+      <c r="G35" s="151" t="n"/>
     </row>
     <row r="36">
-      <c r="F36" s="159" t="n"/>
+      <c r="F36" s="153" t="n"/>
     </row>
     <row r="37">
-      <c r="F37" s="157" t="n"/>
+      <c r="F37" s="151" t="n"/>
     </row>
     <row r="44">
-      <c r="H44" s="160" t="n"/>
+      <c r="H44" s="154" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="18">
     <mergeCell ref="A9:H9"/>
-    <mergeCell ref="A25:C25"/>
     <mergeCell ref="F4:G4"/>
-    <mergeCell ref="A21:H21"/>
-    <mergeCell ref="D28:H28"/>
     <mergeCell ref="F2:H2"/>
     <mergeCell ref="E1:H1"/>
+    <mergeCell ref="A21:E23"/>
+    <mergeCell ref="A25:C27"/>
+    <mergeCell ref="A24:C24"/>
     <mergeCell ref="F3:G3"/>
     <mergeCell ref="D25:H25"/>
     <mergeCell ref="B8:E8"/>
     <mergeCell ref="F6:H6"/>
     <mergeCell ref="C1:D1"/>
+    <mergeCell ref="D24:H24"/>
+    <mergeCell ref="A20:H20"/>
     <mergeCell ref="F5:G5"/>
     <mergeCell ref="D27:H27"/>
-    <mergeCell ref="A26:C28"/>
     <mergeCell ref="F7:H7"/>
-    <mergeCell ref="A22:E24"/>
     <mergeCell ref="D26:H26"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>

</xml_diff>